<commit_message>
added new analyses and modified table
</commit_message>
<xml_diff>
--- a/data/2020-07-24_AgNP-ELA-lakes_fish-excretion.xlsx
+++ b/data/2020-07-24_AgNP-ELA-lakes_fish-excretion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://trentu-my.sharepoint.com/personal/sandraklemet_trentu_ca/Documents/Documents/Etudes/Trent/Xenopoulos lab/Projects/AgNP-ELA_fish-excretion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{CE3E8D6E-5903-41F8-A84F-7FD18A12D88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64A9B145-CB35-4D8C-A758-60E998DFD4E2}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{CE3E8D6E-5903-41F8-A84F-7FD18A12D88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70D62FF7-388D-483E-B3CC-552C958F9D7F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="889" firstSheet="1" activeTab="3" xr2:uid="{33E7FBB4-830F-460A-98F2-8A56863560C3}"/>
+    <workbookView minimized="1" xWindow="37950" yWindow="3615" windowWidth="14400" windowHeight="7545" tabRatio="889" xr2:uid="{33E7FBB4-830F-460A-98F2-8A56863560C3}"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="3" r:id="rId1"/>
@@ -20691,7 +20691,7 @@
         <v>8</v>
       </c>
       <c r="F77" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G77" s="24">
         <v>16</v>
@@ -20810,7 +20810,7 @@
         <v>8</v>
       </c>
       <c r="F78" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G78" s="24">
         <v>16</v>
@@ -20929,7 +20929,7 @@
         <v>8</v>
       </c>
       <c r="F79" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G79" s="24">
         <v>16</v>
@@ -21048,7 +21048,7 @@
         <v>8</v>
       </c>
       <c r="F80" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G80" s="24">
         <v>16</v>
@@ -21165,7 +21165,7 @@
         <v>8</v>
       </c>
       <c r="F81" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G81" s="24">
         <v>16</v>
@@ -21282,7 +21282,7 @@
         <v>8</v>
       </c>
       <c r="F82" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G82" s="24">
         <v>16</v>
@@ -21398,7 +21398,7 @@
         <v>8</v>
       </c>
       <c r="F83" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G83" s="24">
         <v>16</v>
@@ -21517,7 +21517,7 @@
         <v>8</v>
       </c>
       <c r="F84" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G84" s="24">
         <v>16</v>
@@ -21636,7 +21636,7 @@
         <v>8</v>
       </c>
       <c r="F85" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G85" s="24">
         <v>16</v>
@@ -21752,7 +21752,7 @@
         <v>8</v>
       </c>
       <c r="F86" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G86" s="24">
         <v>16</v>
@@ -21871,7 +21871,7 @@
         <v>8</v>
       </c>
       <c r="F87" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G87" s="24">
         <v>16</v>
@@ -21990,7 +21990,7 @@
         <v>8</v>
       </c>
       <c r="F88" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G88" s="24">
         <v>16</v>
@@ -22109,7 +22109,7 @@
         <v>8</v>
       </c>
       <c r="F89" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G89" s="24">
         <v>16</v>
@@ -22228,7 +22228,7 @@
         <v>8</v>
       </c>
       <c r="F90" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G90" s="24">
         <v>16</v>
@@ -22344,7 +22344,7 @@
         <v>8</v>
       </c>
       <c r="F91" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G91" s="24">
         <v>16</v>
@@ -22463,7 +22463,7 @@
         <v>8</v>
       </c>
       <c r="F92" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G92" s="24">
         <v>16</v>
@@ -22580,7 +22580,7 @@
         <v>8</v>
       </c>
       <c r="F93" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G93" s="24">
         <v>16</v>
@@ -22701,7 +22701,7 @@
         <v>8</v>
       </c>
       <c r="F94" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G94" s="24">
         <v>16</v>
@@ -22822,7 +22822,7 @@
         <v>8</v>
       </c>
       <c r="F95" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G95" s="24">
         <v>16</v>
@@ -22943,7 +22943,7 @@
         <v>8</v>
       </c>
       <c r="F96" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G96" s="24">
         <v>16</v>
@@ -23060,7 +23060,7 @@
         <v>8</v>
       </c>
       <c r="F97" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G97" s="24">
         <v>16</v>
@@ -23174,7 +23174,7 @@
         <v>8</v>
       </c>
       <c r="F98" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G98" s="24">
         <v>16</v>
@@ -23288,7 +23288,7 @@
         <v>8</v>
       </c>
       <c r="F99" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G99" s="24">
         <v>16</v>
@@ -23402,7 +23402,7 @@
         <v>8</v>
       </c>
       <c r="F100" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G100" s="24">
         <v>16</v>
@@ -23516,7 +23516,7 @@
         <v>8</v>
       </c>
       <c r="F101" s="25">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G101" s="24">
         <v>16</v>

</xml_diff>